<commit_message>
approver email update add approve | send back
</commit_message>
<xml_diff>
--- a/Documents/devfiles/excel/DevoloperActivities.xlsx
+++ b/Documents/devfiles/excel/DevoloperActivities.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\devfiles\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30CEDFCD-1AB9-44E1-8196-BDDCF2D0366F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC640F5D-0558-4230-A55A-551E710795B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="290" yWindow="860" windowWidth="19000" windowHeight="10510" activeTab="1" xr2:uid="{337275F3-F812-418C-B02B-6398BC7C9B39}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{337275F3-F812-418C-B02B-6398BC7C9B39}"/>
   </bookViews>
   <sheets>
     <sheet name="Draft" sheetId="2" r:id="rId1"/>
     <sheet name="Daily Task" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="6" r:id="rId5"/>
+    <sheet name="ToDo" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="196">
   <si>
     <t>Daily sync of responses from MS forms to be scheduled at: 7AM, 12NN, 3PM</t>
   </si>
@@ -535,12 +537,152 @@
   <si>
     <t>Modal import button Confirmation</t>
   </si>
+  <si>
+    <t>QAS App:</t>
+  </si>
+  <si>
+    <t>10.54.4.28</t>
+  </si>
+  <si>
+    <t>Username: hrappqa_admin</t>
+  </si>
+  <si>
+    <t>Password: $4n#l+0&amp;xg-F&amp;Dfm</t>
+  </si>
+  <si>
+    <t>QAS DB:</t>
+  </si>
+  <si>
+    <t>10.54.4.119</t>
+  </si>
+  <si>
+    <t>Username: hrdbqa_admin</t>
+  </si>
+  <si>
+    <t>Password: SnVyE|4%NsiEyKva</t>
+  </si>
+  <si>
+    <t>HROD Ticketing Tool PROD:</t>
+  </si>
+  <si>
+    <t>Credentials:</t>
+  </si>
+  <si>
+    <t>Database:</t>
+  </si>
+  <si>
+    <t>AEC2HRODTICKETINGDBPROD001 - 10.54.5.69</t>
+  </si>
+  <si>
+    <t>username: hrdb_prod</t>
+  </si>
+  <si>
+    <t>password: $eMAJp%*8&amp;@LgCxn</t>
+  </si>
+  <si>
+    <t>APP:</t>
+  </si>
+  <si>
+    <t>AEC2HRODTICKETINGAPPPROD001 - 10.54.5.46</t>
+  </si>
+  <si>
+    <t>username: hrapp_prod</t>
+  </si>
+  <si>
+    <t>password: zD7C#!CMSjaEyOLK</t>
+  </si>
+  <si>
+    <r>
+      <t>HR JOB OFFER TOOL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>hrjoboffer.unilab.com.ph</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>Add Title Page all Roles/User</t>
+  </si>
+  <si>
+    <t>Import Confirmation message</t>
+  </si>
+  <si>
+    <t>Official Email Subject</t>
+  </si>
+  <si>
+    <t>Notif Bell/Email for Import</t>
+  </si>
+  <si>
+    <t>Proposed - Option 1</t>
+  </si>
+  <si>
+    <t>Remove "Press Enter to Apply"</t>
+  </si>
+  <si>
+    <t>Add Send Back to Email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analysis Auto Compute Annual Allowance </t>
+  </si>
+  <si>
+    <t>Locked Cadidate if it has JO</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>Update the number format of the data coming from MS Forms and Dbox.</t>
+  </si>
+  <si>
+    <t>Match the "Candidate Response" and "Dbox Sync" button</t>
+  </si>
+  <si>
+    <t>Calculate - Annual Values in the Compensation Table based on Monthly</t>
+  </si>
+  <si>
+    <t>Rename the Options - Proposed Option 1; Proposed Option 2</t>
+  </si>
+  <si>
+    <t>Remove - "Press Enter to Apply"</t>
+  </si>
+  <si>
+    <t>Update the spelling of "through" in the email</t>
+  </si>
+  <si>
+    <t>Option tables in the email should be presented horizontally rather than vertically.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -571,8 +713,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -600,6 +749,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -669,7 +824,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -717,6 +872,14 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1238,7 +1401,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EED69CB7-7627-4EC8-B1DF-810A0B37AA79}">
-  <dimension ref="C1:Y26"/>
+  <dimension ref="C1:Y32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.36328125" customWidth="1"/>
@@ -1730,18 +1893,60 @@
       </c>
     </row>
     <row r="23" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H23" s="24" t="s">
+        <v>179</v>
+      </c>
       <c r="I23" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="24" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H24" s="24" t="s">
+        <v>180</v>
+      </c>
       <c r="I24" t="s">
         <v>94</v>
       </c>
     </row>
+    <row r="25" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H25" s="24" t="s">
+        <v>181</v>
+      </c>
+    </row>
     <row r="26" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H26" s="25"/>
       <c r="I26" t="s">
         <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H27" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="28" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H28" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="29" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H29" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="30" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H30" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="31" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H31" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="32" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H32" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -1847,7 +2052,7 @@
       <c r="D3" s="22"/>
       <c r="E3" s="22"/>
     </row>
-    <row r="4" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="17" t="s">
         <v>119</v>
       </c>
@@ -1905,7 +2110,7 @@
       <c r="D9" s="17"/>
       <c r="E9" s="17"/>
     </row>
-    <row r="10" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
         <v>125</v>
       </c>
@@ -1915,7 +2120,7 @@
       <c r="D10" s="22"/>
       <c r="E10" s="22"/>
     </row>
-    <row r="11" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="17" t="s">
         <v>82</v>
       </c>
@@ -1923,7 +2128,7 @@
       <c r="D11" s="22"/>
       <c r="E11" s="22"/>
     </row>
-    <row r="12" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="17" t="s">
         <v>83</v>
       </c>
@@ -1939,7 +2144,7 @@
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
     </row>
-    <row r="14" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B14" s="17" t="s">
         <v>127</v>
       </c>
@@ -1949,7 +2154,7 @@
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
     </row>
-    <row r="15" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="17" t="s">
         <v>128</v>
       </c>
@@ -1981,7 +2186,7 @@
         <v>46286</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B18" s="17" t="s">
         <v>131</v>
       </c>
@@ -2009,7 +2214,7 @@
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
     </row>
-    <row r="21" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="17" t="s">
         <v>133</v>
       </c>
@@ -2025,7 +2230,7 @@
       <c r="D22" s="22"/>
       <c r="E22" s="22"/>
     </row>
-    <row r="23" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="17" t="s">
         <v>134</v>
       </c>
@@ -2033,7 +2238,7 @@
       <c r="D23" s="22"/>
       <c r="E23" s="22"/>
     </row>
-    <row r="24" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="17" t="s">
         <v>135</v>
       </c>
@@ -2041,7 +2246,7 @@
       <c r="D24" s="22"/>
       <c r="E24" s="22"/>
     </row>
-    <row r="25" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="17" t="s">
         <v>136</v>
       </c>
@@ -2049,7 +2254,7 @@
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
     </row>
-    <row r="26" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="17" t="s">
         <v>93</v>
       </c>
@@ -2059,7 +2264,7 @@
       <c r="D26" s="22"/>
       <c r="E26" s="22"/>
     </row>
-    <row r="27" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="17" t="s">
         <v>94</v>
       </c>
@@ -2067,7 +2272,7 @@
       <c r="D27" s="22"/>
       <c r="E27" s="22"/>
     </row>
-    <row r="28" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="17" t="s">
         <v>137</v>
       </c>
@@ -2087,7 +2292,7 @@
       <c r="D29" s="17"/>
       <c r="E29" s="17"/>
     </row>
-    <row r="30" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B30" s="17" t="s">
         <v>139</v>
       </c>
@@ -2097,7 +2302,7 @@
       <c r="D30" s="22"/>
       <c r="E30" s="22"/>
     </row>
-    <row r="31" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="17" t="s">
         <v>140</v>
       </c>
@@ -2105,7 +2310,7 @@
       <c r="D31" s="22"/>
       <c r="E31" s="22"/>
     </row>
-    <row r="32" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="17" t="s">
         <v>141</v>
       </c>
@@ -2113,7 +2318,7 @@
       <c r="D32" s="22"/>
       <c r="E32" s="22"/>
     </row>
-    <row r="33" spans="2:5" ht="58" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
         <v>142</v>
       </c>
@@ -2123,7 +2328,7 @@
       <c r="D33" s="17"/>
       <c r="E33" s="17"/>
     </row>
-    <row r="34" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="17" t="s">
         <v>143</v>
       </c>
@@ -2133,7 +2338,7 @@
       <c r="D34" s="17"/>
       <c r="E34" s="17"/>
     </row>
-    <row r="35" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="17" t="s">
         <v>144</v>
       </c>
@@ -2143,7 +2348,7 @@
       <c r="D35" s="17"/>
       <c r="E35" s="17"/>
     </row>
-    <row r="36" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="17" t="s">
         <v>145</v>
       </c>
@@ -2165,7 +2370,7 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B38" s="17" t="s">
         <v>147</v>
       </c>
@@ -2175,7 +2380,7 @@
       <c r="D38" s="17"/>
       <c r="E38" s="17"/>
     </row>
-    <row r="39" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B39" s="17" t="s">
         <v>148</v>
       </c>
@@ -2185,7 +2390,7 @@
       <c r="D39" s="17"/>
       <c r="E39" s="17"/>
     </row>
-    <row r="40" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B40" s="17" t="s">
         <v>149</v>
       </c>
@@ -2195,7 +2400,7 @@
       <c r="D40" s="17"/>
       <c r="E40" s="17"/>
     </row>
-    <row r="41" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B41" s="17" t="s">
         <v>150</v>
       </c>
@@ -2205,7 +2410,7 @@
       <c r="D41" s="17"/>
       <c r="E41" s="17"/>
     </row>
-    <row r="42" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B42" s="17" t="s">
         <v>151</v>
       </c>
@@ -2227,7 +2432,7 @@
         <v>46296</v>
       </c>
     </row>
-    <row r="44" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B44" s="17" t="s">
         <v>153</v>
       </c>
@@ -2237,7 +2442,7 @@
       <c r="D44" s="17"/>
       <c r="E44" s="17"/>
     </row>
-    <row r="45" spans="2:5" ht="87" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B45" s="17" t="s">
         <v>154</v>
       </c>
@@ -2249,6 +2454,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="E10:E13"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="D30:D32"/>
     <mergeCell ref="E30:E32"/>
@@ -2258,13 +2469,188 @@
     <mergeCell ref="C26:C27"/>
     <mergeCell ref="D26:D27"/>
     <mergeCell ref="E26:E27"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="E10:E13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7A45ED2-CCFB-4370-9B45-2EF1DE8F3431}">
+  <dimension ref="B2:B29"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B17" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B23" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B29" s="23" t="s">
+        <v>178</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F07538F4-CB19-4AAD-A763-90C29763BC37}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="1.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B2" s="17">
+        <v>1</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="17">
+        <v>2</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="17">
+        <v>3</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="17">
+        <v>4</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B6" s="17">
+        <v>5</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B7" s="17">
+        <v>6</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="B8" s="17">
+        <v>7</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>195</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
end of shift commit
</commit_message>
<xml_diff>
--- a/Documents/devfiles/excel/DevoloperActivities.xlsx
+++ b/Documents/devfiles/excel/DevoloperActivities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\devfiles\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B51CA9D9-59BE-4C89-BC80-10BB8C8C2243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{D2130601-5DEE-4F6D-9E84-6E3CC2A0BD64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{337275F3-F812-418C-B02B-6398BC7C9B39}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{337275F3-F812-418C-B02B-6398BC7C9B39}"/>
   </bookViews>
   <sheets>
     <sheet name="Draft" sheetId="2" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="ToDo" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="197">
   <si>
     <t>Daily sync of responses from MS forms to be scheduled at: 7AM, 12NN, 3PM</t>
   </si>
@@ -299,9 +300,6 @@
   </si>
   <si>
     <t>Remove Package Details Table</t>
-  </si>
-  <si>
-    <t>Add Notes Tab under TA Partner access for approval notes from Division Head</t>
   </si>
   <si>
     <t>TA Interface:</t>
@@ -383,9 +381,6 @@
   </si>
   <si>
     <t>cc. Ms. Mariss Ivy D. Batac</t>
-  </si>
-  <si>
-    <t>new password - hrodooffer@1</t>
   </si>
   <si>
     <t>Manual Upload</t>
@@ -676,6 +671,15 @@
   </si>
   <si>
     <t>Option tables in the email should be presented horizontally rather than vertically.</t>
+  </si>
+  <si>
+    <t>Add Notes Tab under TA Partner access for approval notes from Division Head - reused Candidate Feedback to Division Head remarks</t>
+  </si>
+  <si>
+    <t>hrjoboffertool@1</t>
+  </si>
+  <si>
+    <t>new password - hrodooffer@1 | hrjoboffertool@1</t>
   </si>
 </sst>
 </file>
@@ -824,7 +828,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -868,12 +872,6 @@
     <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -882,6 +880,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1410,7 +1418,7 @@
     <col min="4" max="4" width="29.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="63.36328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="46.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="63.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="51.54296875" customWidth="1"/>
     <col min="10" max="10" width="28.90625" customWidth="1"/>
     <col min="11" max="11" width="55.90625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="46.90625" bestFit="1" customWidth="1"/>
@@ -1667,7 +1675,7 @@
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L6" s="10" t="s">
         <v>59</v>
@@ -1681,7 +1689,7 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E7" t="s">
         <v>61</v>
@@ -1693,7 +1701,7 @@
         <v>21</v>
       </c>
       <c r="K7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>60</v>
@@ -1710,13 +1718,13 @@
     </row>
     <row r="8" spans="3:25" x14ac:dyDescent="0.35">
       <c r="D8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I8" t="s">
         <v>22</v>
       </c>
       <c r="K8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O8" s="11" t="s">
         <v>68</v>
@@ -1730,10 +1738,10 @@
     </row>
     <row r="9" spans="3:25" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E9" t="s">
         <v>72</v>
@@ -1742,24 +1750,24 @@
         <v>46</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O9" s="11" t="s">
         <v>69</v>
       </c>
       <c r="Q9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="3:25" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>73</v>
@@ -1771,35 +1779,35 @@
         <v>23</v>
       </c>
       <c r="K10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O10" t="s">
         <v>70</v>
       </c>
       <c r="Q10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="3:25" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="I11" t="s">
         <v>24</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O11" s="11" t="s">
         <v>46</v>
       </c>
       <c r="Q11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="3:25" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E12" t="s">
         <v>74</v>
@@ -1811,9 +1819,9 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="3:25" x14ac:dyDescent="0.35">
+    <row r="13" spans="3:25" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E13" t="s">
         <v>75</v>
@@ -1821,8 +1829,8 @@
       <c r="H13" t="s">
         <v>39</v>
       </c>
-      <c r="I13" t="s">
-        <v>85</v>
+      <c r="I13" s="25" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="14" spans="3:25" x14ac:dyDescent="0.35">
@@ -1838,7 +1846,7 @@
         <v>77</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="3:25" x14ac:dyDescent="0.35">
@@ -1849,7 +1857,7 @@
         <v>80</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="5:9" x14ac:dyDescent="0.35">
@@ -1857,7 +1865,7 @@
         <v>79</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="5:9" x14ac:dyDescent="0.35">
@@ -1865,7 +1873,7 @@
         <v>81</v>
       </c>
       <c r="I18" s="12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="5:9" x14ac:dyDescent="0.35">
@@ -1873,7 +1881,7 @@
         <v>82</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="5:9" x14ac:dyDescent="0.35">
@@ -1881,7 +1889,7 @@
         <v>83</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="5:9" x14ac:dyDescent="0.35">
@@ -1889,64 +1897,64 @@
         <v>84</v>
       </c>
       <c r="I21" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H23" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="I23" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="5:9" x14ac:dyDescent="0.35">
-      <c r="H23" s="24" t="s">
+    <row r="24" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H24" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="I24" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="25" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H25" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="I23" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="24" spans="5:9" x14ac:dyDescent="0.35">
-      <c r="H24" s="24" t="s">
-        <v>180</v>
-      </c>
-      <c r="I24" t="s">
+    </row>
+    <row r="26" spans="5:9" x14ac:dyDescent="0.35">
+      <c r="H26" s="23"/>
+      <c r="I26" t="s">
         <v>94</v>
-      </c>
-    </row>
-    <row r="25" spans="5:9" x14ac:dyDescent="0.35">
-      <c r="H25" s="24" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="26" spans="5:9" x14ac:dyDescent="0.35">
-      <c r="H26" s="25"/>
-      <c r="I26" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="27" spans="5:9" x14ac:dyDescent="0.35">
       <c r="H27" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="5:9" x14ac:dyDescent="0.35">
       <c r="H28" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="29" spans="5:9" x14ac:dyDescent="0.35">
       <c r="H29" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="5:9" x14ac:dyDescent="0.35">
       <c r="H30" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="5:9" x14ac:dyDescent="0.35">
       <c r="H31" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="32" spans="5:9" x14ac:dyDescent="0.35">
       <c r="H32" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -1956,55 +1964,59 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19B8C298-1B1E-4BB2-871B-BB0A034CE40B}">
-  <dimension ref="B2:B14"/>
+  <dimension ref="B2:C14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="123.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B2" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="15" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B3" s="15" t="s">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B4" s="15" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B4" s="15" t="s">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="14" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B5" s="14" t="s">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B6" s="12" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B6" s="12" t="s">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B7" s="16" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B7" s="16" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>109</v>
+        <v>196</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -2012,6 +2024,7 @@
     <hyperlink ref="B3" r:id="rId1" display="mailto:HRODJobOffer1@unilab.com.ph" xr:uid="{91CE123A-88F9-43A8-B644-9987241107B6}"/>
     <hyperlink ref="B4" r:id="rId2" display="mailto:HRODJobOffer2@unilab.com.ph" xr:uid="{F1C187EC-B40B-4FAE-A673-CEEE66EDB502}"/>
     <hyperlink ref="B7" r:id="rId3" display="mailto:mdbatac@unilab.com.ph" xr:uid="{8910D44C-91EB-49B4-8102-31F5ACADA21E}"/>
+    <hyperlink ref="C14" r:id="rId4" xr:uid="{F86505C5-C7F3-41A3-9C5C-FA7382175A2A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2030,10 +2043,10 @@
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B2" s="18" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D2" s="20">
         <v>46273</v>
@@ -2044,25 +2057,25 @@
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="C3" s="21">
+        <v>116</v>
+      </c>
+      <c r="C3" s="26">
         <v>46274</v>
       </c>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-    </row>
-    <row r="5" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+      <c r="C4" s="26"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" s="17" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C5" s="19">
         <v>46275</v>
@@ -2070,9 +2083,9 @@
       <c r="D5" s="17"/>
       <c r="E5" s="17"/>
     </row>
-    <row r="6" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="17" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C6" s="19">
         <v>46276</v>
@@ -2080,9 +2093,9 @@
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
     </row>
-    <row r="7" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="17" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C7" s="19">
         <v>46276</v>
@@ -2090,9 +2103,9 @@
       <c r="D7" s="17"/>
       <c r="E7" s="17"/>
     </row>
-    <row r="8" spans="2:5" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B8" s="17" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C8" s="19">
         <v>46279</v>
@@ -2100,9 +2113,9 @@
       <c r="D8" s="17"/>
       <c r="E8" s="17"/>
     </row>
-    <row r="9" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="17" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C9" s="19">
         <v>46279</v>
@@ -2112,41 +2125,41 @@
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="C10" s="21">
+        <v>123</v>
+      </c>
+      <c r="C10" s="26">
         <v>46279</v>
       </c>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
+        <v>124</v>
+      </c>
+      <c r="C13" s="26"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
     </row>
     <row r="14" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B14" s="17" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C14" s="19">
         <v>46279</v>
@@ -2156,7 +2169,7 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="17" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C15" s="19">
         <v>46279</v>
@@ -2166,7 +2179,7 @@
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C16" s="19">
         <v>46279</v>
@@ -2176,7 +2189,7 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="20">
@@ -2188,7 +2201,7 @@
     </row>
     <row r="18" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B18" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C18" s="19">
         <v>46280</v>
@@ -2198,83 +2211,83 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="C19" s="21">
+        <v>130</v>
+      </c>
+      <c r="C19" s="26">
         <v>46280</v>
       </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="C20" s="21"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
+        <v>86</v>
+      </c>
+      <c r="C20" s="26"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="C21" s="21"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
+        <v>131</v>
+      </c>
+      <c r="C21" s="26"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" s="21"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
+        <v>88</v>
+      </c>
+      <c r="C22" s="26"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="C23" s="21"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
+        <v>132</v>
+      </c>
+      <c r="C23" s="26"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
+        <v>133</v>
+      </c>
+      <c r="C24" s="26"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
+        <v>134</v>
+      </c>
+      <c r="C25" s="26"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="C26" s="21">
+        <v>92</v>
+      </c>
+      <c r="C26" s="26">
         <v>46280</v>
       </c>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="C27" s="21"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
+        <v>93</v>
+      </c>
+      <c r="C27" s="26"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="17" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C28" s="19">
         <v>46280</v>
@@ -2284,7 +2297,7 @@
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="17" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C29" s="19">
         <v>46281</v>
@@ -2294,33 +2307,33 @@
     </row>
     <row r="30" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B30" s="17" t="s">
-        <v>139</v>
-      </c>
-      <c r="C30" s="21">
+        <v>137</v>
+      </c>
+      <c r="C30" s="26">
         <v>46282</v>
       </c>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="C31" s="21"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
+        <v>138</v>
+      </c>
+      <c r="C31" s="26"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
+        <v>139</v>
+      </c>
+      <c r="C32" s="26"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
     </row>
     <row r="33" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C33" s="19">
         <v>46283</v>
@@ -2330,7 +2343,7 @@
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="17" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C34" s="19">
         <v>46283</v>
@@ -2340,7 +2353,7 @@
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="17" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C35" s="19">
         <v>46286</v>
@@ -2350,7 +2363,7 @@
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C36" s="19">
         <v>46286</v>
@@ -2360,7 +2373,7 @@
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B37" s="17" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C37" s="17"/>
       <c r="D37" s="19">
@@ -2372,7 +2385,7 @@
     </row>
     <row r="38" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B38" s="17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C38" s="19">
         <v>46287</v>
@@ -2382,7 +2395,7 @@
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B39" s="17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C39" s="19">
         <v>46288</v>
@@ -2392,7 +2405,7 @@
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B40" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C40" s="19">
         <v>46289</v>
@@ -2402,7 +2415,7 @@
     </row>
     <row r="41" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B41" s="17" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C41" s="19">
         <v>46289</v>
@@ -2412,7 +2425,7 @@
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B42" s="17" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C42" s="19">
         <v>46290</v>
@@ -2422,7 +2435,7 @@
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B43" s="18" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C43" s="17"/>
       <c r="D43" s="20">
@@ -2434,7 +2447,7 @@
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B44" s="17" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C44" s="19">
         <v>46294</v>
@@ -2444,7 +2457,7 @@
     </row>
     <row r="45" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B45" s="17" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C45" s="19">
         <v>46296</v>
@@ -2454,12 +2467,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="E10:E13"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="D30:D32"/>
     <mergeCell ref="E30:E32"/>
@@ -2469,6 +2476,12 @@
     <mergeCell ref="C26:C27"/>
     <mergeCell ref="D26:D27"/>
     <mergeCell ref="E26:E27"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="E10:E13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2481,97 +2494,97 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B23" s="1" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B29" s="23" t="s">
-        <v>178</v>
+      <c r="B29" s="21" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -2591,23 +2604,23 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B2" s="17">
         <v>1</v>
       </c>
-      <c r="C2" s="26" t="s">
-        <v>189</v>
+      <c r="C2" s="24" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B3" s="17">
         <v>2</v>
       </c>
-      <c r="C3" s="26" t="s">
-        <v>190</v>
+      <c r="C3" s="24" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -2615,31 +2628,31 @@
         <v>3</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B5" s="17">
         <v>4</v>
       </c>
-      <c r="C5" s="26" t="s">
-        <v>192</v>
+      <c r="C5" s="24" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B6" s="17">
         <v>5</v>
       </c>
-      <c r="C6" s="26" t="s">
-        <v>193</v>
+      <c r="C6" s="24" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B7" s="17">
         <v>6</v>
       </c>
-      <c r="C7" s="26" t="s">
-        <v>194</v>
+      <c r="C7" s="24" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -2647,7 +2660,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>